<commit_message>
Add official-sources checklist to matrix and Delphi round 1 questionnaire
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QKbj24VsGxk6d97XVHWeWi
</commit_message>
<xml_diff>
--- a/cyber_audit_component_matrix.xlsx
+++ b/cyber_audit_component_matrix.xlsx
@@ -11,7 +11,8 @@
     <sheet name="راهنما" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="ماتریس" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="اصلاح_ارجاعات" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="مقایسه_دو_گروه" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="منابع_رسمی" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="مقایسه_دو_گروه" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">ماتریس!$A$4:$M$34</definedName>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="368">
   <si>
     <t xml:space="preserve">ماتریس مولفه‌های ارزیابی ریسک سایبری توسط حسابرسان – پیش‌نویس مرحله اول پژوهش</t>
   </si>
@@ -79,7 +80,7 @@
     <t xml:space="preserve">ماتریس نگاشت مولفه‌های ارزیابی ریسک سایبری در حسابرسی: دیدگاه سازمان و دیدگاه حسابرس</t>
   </si>
   <si>
-    <t xml:space="preserve">توجه: همه ارجاع‌ها پیش‌نویس هستند و باید پیش از استفاده در مقاله با متن رسمی استاندارد/چارچوب تطبیق داده شوند (ستون «وضعیت راستی‌آزمایی»). ستون «پیشینه پژوهش» را خودتان پر کنید.</t>
+    <t xml:space="preserve">توجه: ارجاع‌ها فقط تا حدی با منابع ثانویه کنترل شده‌اند (ساختار NIST CSF 2.0، ISO 27002:2022 و TSC) و شماره دقیق بندها باید با متن رسمی در شیت «منابع_رسمی» تطبیق و تیک بخورد. ستون «پیشینه پژوهش» را خودتان پر کنید.</t>
   </si>
   <si>
     <t xml:space="preserve">کد</t>
@@ -148,7 +149,7 @@
     <t xml:space="preserve">ISA 315 (Revised 2019) – درک محیط کنترلی; ISA 260</t>
   </si>
   <si>
-    <t xml:space="preserve">نیاز به تطبیق با متن رسمی</t>
+    <t xml:space="preserve">ساختار با منابع ثانویه سازگار؛ بند/زیرمعیار دقیق هنوز با متن رسمی تطبیق نشده</t>
   </si>
   <si>
     <t xml:space="preserve">C02</t>
@@ -935,6 +936,171 @@
   </si>
   <si>
     <t xml:space="preserve">ارجاع کلی کافی نیست؛ بند/کنترل دقیق بنویسید.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فهرست منابع رسمی برای تطبیق ارجاع‌ها (قبل از ارسال مقاله هر مورد باید با متن اصلی چک و تیک بخورد)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">منبع (به سبک مرجع‌نویسی)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ناشر</t>
+  </si>
+  <si>
+    <t xml:space="preserve">نشانی رسمی برای دریافت</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تطبیق شد؟ (بله/خیر)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">نکته</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AICPA. (2017). 2017 Trust Services Criteria for Security, Availability, Processing Integrity, Confidentiality, and Privacy (With Revised Points of Focus—2022). TSP Section 100.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AICPA &amp; CIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aicpa-cima.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">معیارهای CC1 تا CC9، A1، C1، PI1، P1–P8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AICPA. (2017). Description Criteria for Management's Description of an Entity's Cybersecurity Risk Management Program (DC Section 100).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مبنای SOC for Cybersecurity؛ شماره DC200 را تطبیق دهید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AICPA. SOC for Cybersecurity – Guide: Reporting on an Entity's Cybersecurity Risk Management Program and Controls.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ویرایش و سال را از سایت ثبت کنید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIST. (2024). The NIST Cybersecurity Framework (CSF) 2.0 (NIST CSWP 29). https://doi.org/10.6028/NIST.CSWP.29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nist.gov / doi.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functions: GV, ID, PR, DE, RS, RC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIST. (2012). Guide for Conducting Risk Assessments (SP 800-30 Rev. 1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">csrc.nist.gov</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIST. (2025). Incident Response Recommendations and Considerations for Cybersecurity Risk Management: A CSF 2.0 Community Profile (SP 800-61 Rev. 3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">جایگزین Rev. 2؛ عنوان و تاریخ را تطبیق دهید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NIST. (2006). Guide to Computer Security Log Management (SP 800-92).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">بررسی کنید ویرایش جدیدتر منتشر نشده باشد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO/IEC. (2022). ISO/IEC 27001:2022 Information security, cybersecurity and privacy protection — Information security management systems — Requirements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO/IEC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iso.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">بندهای 4 تا 10 و Annex A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO/IEC. (2022). ISO/IEC 27002:2022 Information security controls.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93 کنترل در 4 گروه؛ شماره کنترل‌ها را از متن تطبیق دهید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO/IEC. (2022). ISO/IEC 27005:2022 Guidance on managing information security risks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">در ماتریس شماره بند آورده نشده؛ در صورت نیاز از متن اضافه شود</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO/IEC. ISO/IEC 27031 (Business continuity ICT readiness) – ویرایش جاری.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سال آخرین ویرایش را تطبیق دهید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO/IEC. ISO/IEC 27036-1 (Supplier relationships) – ویرایش جاری.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO/IEC. ISO/IEC 29134 (Guidelines for privacy impact assessment) – ویرایش جاری.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">جایگزین ارجاع نادرست 29100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO. (2018). ISO 31000:2018 Risk management — Guidelines. / IEC 31010:2019 Risk assessment techniques.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO / IEC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISO/IEC. ISO/IEC 27034-1 Application security – Overview and concepts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سال/ویرایش را تطبیق دهید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAASB. International Standard on Auditing 315 (Revised 2019), Identifying and Assessing the Risks of Material Misstatement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAASB / IFAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iaasb.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ارجاع به بندهای مربوط به درک محیط IT را از متن اضافه کنید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAASB. ISA 200, 230, 240, 250, 260, 265, 330, 402, 450, 500, 560, 570, 620 و ISQM 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ویرایش‌های جاری (به‌ویژه 570 و 220) را چک کنید</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCAOB. AS 2110 Identifying and Assessing Risks of Material Misstatement; AS 2201 An Audit of Internal Control Over Financial Reporting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCAOB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pcaobus.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فقط اگر دیدگاه آمریکایی لازم است</t>
+  </si>
+  <si>
+    <t xml:space="preserve">استانداردهای حسابرسی ایران (ترجمه/تطبیق ISA) – ویرایش جاری</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سازمان حسابرسی</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مرجع رسمی سازمان حسابرسی</t>
+  </si>
+  <si>
+    <t xml:space="preserve">شماره و نسخه ایرانی ISAها را از متن رسمی تطبیق دهید</t>
   </si>
   <si>
     <t xml:space="preserve">ابزار مقایسه اهمیت مولفه‌ها از دید دو گروه: سازمان مورد رسیدگی و حسابرسان</t>
@@ -3256,6 +3422,396 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="E4" s="9"/>
+      <c r="F4" s="4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="E5" s="9"/>
+      <c r="F5" s="4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="4" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="4" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="E8" s="9"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="E9" s="9"/>
+      <c r="F9" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="E10" s="9"/>
+      <c r="F10" s="4" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="4" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E12" s="9"/>
+      <c r="F12" s="4" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E13" s="9"/>
+      <c r="F13" s="4" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E14" s="9"/>
+      <c r="F14" s="4" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="4" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E16" s="9"/>
+      <c r="F16" s="4" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E17" s="9"/>
+      <c r="F17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="E18" s="9"/>
+      <c r="F18" s="4" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="E19" s="9"/>
+      <c r="F19" s="4" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="E20" s="9"/>
+      <c r="F20" s="4" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="E21" s="9"/>
+      <c r="F21" s="4" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="E22" s="9"/>
+      <c r="F22" s="4" t="s">
+        <v>357</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3269,12 +3825,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>303</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>304</v>
+        <v>359</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -3283,12 +3839,12 @@
         <v>1</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>305</v>
+        <v>360</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="11.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>306</v>
+        <v>361</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="15"/>
@@ -3308,24 +3864,24 @@
         <v>22</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>307</v>
+        <v>362</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>308</v>
+        <v>363</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>309</v>
+        <v>364</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>311</v>
+        <v>366</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>312</v>
+        <v>367</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
Add theory, hypotheses and novelty documents (fa/en), reference verification report; fix SOC for Cybersecurity DC reference in matrix
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QKbj24VsGxk6d97XVHWeWi
</commit_message>
<xml_diff>
--- a/cyber_audit_component_matrix.xlsx
+++ b/cyber_audit_component_matrix.xlsx
@@ -185,7 +185,7 @@
     <t xml:space="preserve">مشترک</t>
   </si>
   <si>
-    <t xml:space="preserve">CC3.1; توصیف سیستم (DC200 در SOC for Cybersecurity)</t>
+    <t xml:space="preserve">CC3.1; SOC for Cybersecurity: DC section 100 (معیارهای توصیف برنامه مدیریت ریسک سایبری)</t>
   </si>
   <si>
     <t xml:space="preserve">GV.OC</t>
@@ -971,7 +971,7 @@
     <t xml:space="preserve">AICPA. (2017). Description Criteria for Management's Description of an Entity's Cybersecurity Risk Management Program (DC Section 100).</t>
   </si>
   <si>
-    <t xml:space="preserve">مبنای SOC for Cybersecurity؛ شماره DC200 را تطبیق دهید</t>
+    <t xml:space="preserve">DC section 100 (تأییدشده با جست‌وجو؛ DC 200 مربوط به SOC 2 است)</t>
   </si>
   <si>
     <t xml:space="preserve">AICPA. SOC for Cybersecurity – Guide: Reporting on an Entity's Cybersecurity Risk Management Program and Controls.</t>

</xml_diff>